<commit_message>
Removed unwanted files and resolved login issue
</commit_message>
<xml_diff>
--- a/pds_admin_mizoram/Backend/Backend/Data_3.xlsx
+++ b/pds_admin_mizoram/Backend/Backend/Data_3.xlsx
@@ -895,10 +895,10 @@
         <v>5000</v>
       </c>
       <c r="K2">
-        <v>765.76</v>
+        <v>721.89</v>
       </c>
       <c r="L2">
-        <v>4234.24</v>
+        <v>4278.11</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -1156,10 +1156,10 @@
         <v>3000</v>
       </c>
       <c r="K11">
-        <v>2986.01</v>
+        <v>2992.06</v>
       </c>
       <c r="L11">
-        <v>13.98999999999978</v>
+        <v>7.940000000000055</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1243,10 +1243,10 @@
         <v>7500</v>
       </c>
       <c r="K14">
-        <v>7495.08</v>
+        <v>7499.62</v>
       </c>
       <c r="L14">
-        <v>4.920000000000073</v>
+        <v>0.3800000000001091</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1272,10 +1272,10 @@
         <v>5000</v>
       </c>
       <c r="K15">
-        <v>4999.37</v>
+        <v>4999.72</v>
       </c>
       <c r="L15">
-        <v>0.6300000000001091</v>
+        <v>0.2799999999997453</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1301,10 +1301,10 @@
         <v>5000</v>
       </c>
       <c r="K16">
-        <v>4997.61</v>
+        <v>4995.29</v>
       </c>
       <c r="L16">
-        <v>2.390000000000327</v>
+        <v>4.710000000000036</v>
       </c>
     </row>
     <row r="17" spans="2:12">
@@ -1504,10 +1504,10 @@
         <v>2000</v>
       </c>
       <c r="K23">
-        <v>1138.71</v>
+        <v>1173.96</v>
       </c>
       <c r="L23">
-        <v>861.29</v>
+        <v>826.04</v>
       </c>
     </row>
     <row r="24" spans="2:12">

</xml_diff>